<commit_message>
Atualização automática: reajuste (15/09/2026 08:58)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,8 +329,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -354,12 +362,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,13 +685,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1274,37 +1300,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1327,13 +1353,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1356,13 +1382,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1391,13 +1417,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1420,13 +1446,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1455,13 +1481,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1490,13 +1516,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1519,13 +1545,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1548,13 +1574,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1577,13 +1603,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1609,13 +1635,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1644,13 +1670,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1673,13 +1699,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1708,13 +1734,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1737,13 +1763,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1772,13 +1798,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1807,13 +1833,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1828,24 +1854,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1862,7 +1888,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1879,7 +1905,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1896,7 +1922,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1913,7 +1939,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1930,7 +1956,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1947,7 +1973,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1964,7 +1990,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -1981,7 +2007,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -1998,7 +2024,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2015,7 +2041,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2032,7 +2058,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2049,7 +2075,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2066,7 +2092,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2083,7 +2109,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2100,7 +2126,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2117,7 +2143,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2134,7 +2160,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2151,7 +2177,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2168,7 +2194,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2185,7 +2211,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2202,7 +2228,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2219,7 +2245,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2236,7 +2262,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2253,7 +2279,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2270,7 +2296,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2287,7 +2313,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2304,7 +2330,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2321,7 +2347,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2338,7 +2364,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2355,7 +2381,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2372,7 +2398,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2389,7 +2415,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2406,7 +2432,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2423,7 +2449,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2440,7 +2466,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2457,7 +2483,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2474,7 +2500,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2491,7 +2517,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2508,7 +2534,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2525,7 +2551,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2542,7 +2568,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2559,7 +2585,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2576,7 +2602,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2593,7 +2619,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2610,7 +2636,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2627,7 +2653,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2644,7 +2670,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2661,7 +2687,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2678,7 +2704,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2695,7 +2721,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2712,7 +2738,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2729,7 +2755,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2746,7 +2772,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2763,7 +2789,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2780,7 +2806,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2797,7 +2823,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2824,16 +2850,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (15/09/2026 12:34)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,16 +329,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -354,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -362,30 +354,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -685,13 +659,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1300,37 +1274,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1353,13 +1327,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1382,13 +1356,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1417,13 +1391,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1446,13 +1420,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1481,13 +1455,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1516,13 +1490,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1545,13 +1519,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1574,13 +1548,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1603,13 +1577,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1635,13 +1609,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1670,13 +1644,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1699,13 +1673,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1734,13 +1708,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1763,13 +1737,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1798,13 +1772,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1833,13 +1807,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1854,24 +1828,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1888,7 +1862,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1905,7 +1879,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1922,7 +1896,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1939,7 +1913,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1956,7 +1930,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1973,7 +1947,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1990,7 +1964,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2007,7 +1981,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2024,7 +1998,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2041,7 +2015,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2058,7 +2032,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2075,7 +2049,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2092,7 +2066,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2109,7 +2083,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2126,7 +2100,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2143,7 +2117,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2160,7 +2134,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2177,7 +2151,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2194,7 +2168,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2211,7 +2185,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2228,7 +2202,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2245,7 +2219,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2262,7 +2236,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2279,7 +2253,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2296,7 +2270,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2313,7 +2287,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2330,7 +2304,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2347,7 +2321,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2364,7 +2338,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2381,7 +2355,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2398,7 +2372,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2415,7 +2389,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2432,7 +2406,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2449,7 +2423,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2466,7 +2440,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2483,7 +2457,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2500,7 +2474,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2517,7 +2491,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2534,7 +2508,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2551,7 +2525,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2568,7 +2542,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2585,7 +2559,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2602,7 +2576,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2619,7 +2593,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2636,7 +2610,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2653,7 +2627,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2670,7 +2644,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2687,7 +2661,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2704,7 +2678,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2721,7 +2695,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2738,7 +2712,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2755,7 +2729,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2772,7 +2746,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2789,7 +2763,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2806,7 +2780,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2823,7 +2797,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2850,16 +2824,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (15/09/2026 14:03)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,8 +329,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -354,12 +362,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,13 +685,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1274,37 +1300,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1327,13 +1353,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1356,13 +1382,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1391,13 +1417,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1420,13 +1446,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1455,13 +1481,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1490,13 +1516,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1519,13 +1545,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1548,13 +1574,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1577,13 +1603,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1609,13 +1635,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1644,13 +1670,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1673,13 +1699,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1708,13 +1734,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1737,13 +1763,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1772,13 +1798,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1807,13 +1833,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1828,24 +1854,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1862,7 +1888,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1879,7 +1905,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1896,7 +1922,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1913,7 +1939,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1930,7 +1956,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1947,7 +1973,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1964,7 +1990,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -1981,7 +2007,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -1998,7 +2024,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2015,7 +2041,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2032,7 +2058,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2049,7 +2075,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2066,7 +2092,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2083,7 +2109,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2100,7 +2126,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2117,7 +2143,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2134,7 +2160,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2151,7 +2177,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2168,7 +2194,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2185,7 +2211,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2202,7 +2228,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2219,7 +2245,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2236,7 +2262,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2253,7 +2279,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2270,7 +2296,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2287,7 +2313,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2304,7 +2330,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2321,7 +2347,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2338,7 +2364,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2355,7 +2381,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2372,7 +2398,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2389,7 +2415,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2406,7 +2432,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2423,7 +2449,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2440,7 +2466,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2457,7 +2483,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2474,7 +2500,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2491,7 +2517,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2508,7 +2534,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2525,7 +2551,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2542,7 +2568,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2559,7 +2585,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2576,7 +2602,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2593,7 +2619,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2610,7 +2636,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2627,7 +2653,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2644,7 +2670,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2661,7 +2687,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2678,7 +2704,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2695,7 +2721,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2712,7 +2738,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2729,7 +2755,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2746,7 +2772,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2763,7 +2789,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2780,7 +2806,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2797,7 +2823,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2824,16 +2850,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (16/09/2026 12:26)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,16 +329,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -354,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -362,30 +354,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -685,13 +659,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1300,37 +1274,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1353,13 +1327,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1382,13 +1356,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1417,13 +1391,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1446,13 +1420,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1481,13 +1455,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1516,13 +1490,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1545,13 +1519,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1574,13 +1548,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1603,13 +1577,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1635,13 +1609,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1670,13 +1644,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1699,13 +1673,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1734,13 +1708,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1763,13 +1737,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1798,13 +1772,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1833,13 +1807,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1854,24 +1828,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1888,7 +1862,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1905,7 +1879,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1922,7 +1896,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1939,7 +1913,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1956,7 +1930,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1973,7 +1947,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1990,7 +1964,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2007,7 +1981,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2024,7 +1998,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2041,7 +2015,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2058,7 +2032,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2075,7 +2049,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2092,7 +2066,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2109,7 +2083,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2126,7 +2100,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2143,7 +2117,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2160,7 +2134,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2177,7 +2151,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2194,7 +2168,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2211,7 +2185,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2228,7 +2202,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2245,7 +2219,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2262,7 +2236,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2279,7 +2253,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2296,7 +2270,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2313,7 +2287,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2330,7 +2304,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2347,7 +2321,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2364,7 +2338,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2381,7 +2355,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2398,7 +2372,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2415,7 +2389,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2432,7 +2406,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2449,7 +2423,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2466,7 +2440,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2483,7 +2457,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2500,7 +2474,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2517,7 +2491,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2534,7 +2508,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2551,7 +2525,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2568,7 +2542,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2585,7 +2559,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2602,7 +2576,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2619,7 +2593,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2636,7 +2610,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2653,7 +2627,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2670,7 +2644,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2687,7 +2661,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2704,7 +2678,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2721,7 +2695,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2738,7 +2712,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2755,7 +2729,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2772,7 +2746,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2789,7 +2763,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2806,7 +2780,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2823,7 +2797,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2850,16 +2824,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (16/09/2026 12:43)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,8 +329,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -354,12 +362,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,13 +685,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1274,37 +1300,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1327,13 +1353,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1356,13 +1382,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1391,13 +1417,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1420,13 +1446,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1455,13 +1481,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1490,13 +1516,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1519,13 +1545,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1548,13 +1574,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1577,13 +1603,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1609,13 +1635,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1644,13 +1670,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1673,13 +1699,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1708,13 +1734,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1737,13 +1763,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1772,13 +1798,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1807,13 +1833,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1828,24 +1854,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1862,7 +1888,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1879,7 +1905,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1896,7 +1922,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1913,7 +1939,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1930,7 +1956,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1947,7 +1973,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1964,7 +1990,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -1981,7 +2007,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -1998,7 +2024,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2015,7 +2041,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2032,7 +2058,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2049,7 +2075,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2066,7 +2092,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2083,7 +2109,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2100,7 +2126,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2117,7 +2143,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2134,7 +2160,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2151,7 +2177,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2168,7 +2194,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2185,7 +2211,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2202,7 +2228,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2219,7 +2245,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2236,7 +2262,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2253,7 +2279,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2270,7 +2296,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2287,7 +2313,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2304,7 +2330,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2321,7 +2347,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2338,7 +2364,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2355,7 +2381,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2372,7 +2398,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2389,7 +2415,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2406,7 +2432,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2423,7 +2449,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2440,7 +2466,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2457,7 +2483,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2474,7 +2500,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2491,7 +2517,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2508,7 +2534,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2525,7 +2551,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2542,7 +2568,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2559,7 +2585,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2576,7 +2602,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2593,7 +2619,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2610,7 +2636,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2627,7 +2653,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2644,7 +2670,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2661,7 +2687,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2678,7 +2704,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2695,7 +2721,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2712,7 +2738,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2729,7 +2755,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2746,7 +2772,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2763,7 +2789,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2780,7 +2806,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2797,7 +2823,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2824,16 +2850,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (17/09/2026 12:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,16 +329,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -354,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -362,30 +354,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -685,13 +659,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1038,7 +1012,7 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B33" t="s">
         <v>27</v>
@@ -1049,7 +1023,7 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B34" t="s">
         <v>3</v>
@@ -1060,7 +1034,7 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B35" t="s">
         <v>4</v>
@@ -1071,7 +1045,7 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B36" t="s">
         <v>5</v>
@@ -1082,7 +1056,7 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B37" t="s">
         <v>28</v>
@@ -1093,7 +1067,7 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B38" t="s">
         <v>29</v>
@@ -1104,7 +1078,7 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B39" t="s">
         <v>30</v>
@@ -1115,7 +1089,7 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B40" t="s">
         <v>31</v>
@@ -1126,7 +1100,7 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B41" t="s">
         <v>12</v>
@@ -1137,7 +1111,7 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B42" t="s">
         <v>13</v>
@@ -1148,7 +1122,7 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B43" t="s">
         <v>14</v>
@@ -1159,7 +1133,7 @@
     </row>
     <row r="44" spans="1:3">
       <c r="A44">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B44" t="s">
         <v>15</v>
@@ -1170,7 +1144,7 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B45" t="s">
         <v>16</v>
@@ -1181,7 +1155,7 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B46" t="s">
         <v>17</v>
@@ -1192,7 +1166,7 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B47" t="s">
         <v>18</v>
@@ -1203,7 +1177,7 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B48" t="s">
         <v>32</v>
@@ -1214,7 +1188,7 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B49" t="s">
         <v>33</v>
@@ -1225,7 +1199,7 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B50" t="s">
         <v>34</v>
@@ -1236,7 +1210,7 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B51" t="s">
         <v>35</v>
@@ -1247,7 +1221,7 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B52" t="s">
         <v>36</v>
@@ -1258,7 +1232,7 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B53" t="s">
         <v>24</v>
@@ -1269,7 +1243,7 @@
     </row>
     <row r="54" spans="1:3">
       <c r="A54">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B54" t="s">
         <v>25</v>
@@ -1280,7 +1254,7 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B55" t="s">
         <v>37</v>
@@ -1300,37 +1274,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1353,13 +1327,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1382,13 +1356,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1417,13 +1391,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1446,13 +1420,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1481,13 +1455,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1516,13 +1490,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1545,13 +1519,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1574,13 +1548,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1603,13 +1577,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1635,13 +1609,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1670,13 +1644,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1699,13 +1673,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1734,13 +1708,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1763,13 +1737,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1798,13 +1772,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1833,13 +1807,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1854,24 +1828,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1888,7 +1862,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1905,7 +1879,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1922,7 +1896,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1939,7 +1913,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1956,7 +1930,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1973,7 +1947,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1990,7 +1964,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2007,7 +1981,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2024,7 +1998,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2041,7 +2015,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2058,7 +2032,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2075,7 +2049,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2092,7 +2066,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2109,7 +2083,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2126,7 +2100,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2143,7 +2117,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2160,7 +2134,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2177,7 +2151,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2194,7 +2168,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2211,7 +2185,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2228,7 +2202,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2245,7 +2219,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2262,7 +2236,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2279,7 +2253,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2296,7 +2270,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2313,7 +2287,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2330,7 +2304,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2347,7 +2321,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2364,7 +2338,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2381,7 +2355,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2398,7 +2372,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2415,7 +2389,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2432,7 +2406,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2449,7 +2423,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2466,7 +2440,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2483,7 +2457,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2500,7 +2474,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2517,7 +2491,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2534,7 +2508,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2551,7 +2525,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2568,7 +2542,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2585,7 +2559,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2602,7 +2576,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2619,7 +2593,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2636,7 +2610,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2653,7 +2627,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2670,7 +2644,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2687,7 +2661,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2704,7 +2678,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2721,7 +2695,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2738,7 +2712,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2755,7 +2729,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2772,7 +2746,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2789,7 +2763,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2806,7 +2780,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2823,7 +2797,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2850,16 +2824,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (17/09/2026 13:00)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,8 +329,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -354,12 +362,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,13 +685,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1274,37 +1300,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1327,13 +1353,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1356,13 +1382,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1391,13 +1417,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1420,13 +1446,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1455,13 +1481,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1490,13 +1516,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1519,13 +1545,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1548,13 +1574,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1577,13 +1603,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1609,13 +1635,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1644,13 +1670,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1673,13 +1699,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1708,13 +1734,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1737,13 +1763,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1772,13 +1798,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1807,13 +1833,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1828,24 +1854,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1862,7 +1888,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1879,7 +1905,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1896,7 +1922,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1913,7 +1939,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1930,7 +1956,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1947,7 +1973,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1964,7 +1990,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -1981,7 +2007,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -1998,7 +2024,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2015,7 +2041,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2032,7 +2058,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2049,7 +2075,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2066,7 +2092,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2083,7 +2109,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2100,7 +2126,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2117,7 +2143,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2134,7 +2160,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2151,7 +2177,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2168,7 +2194,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2185,7 +2211,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2202,7 +2228,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2219,7 +2245,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2236,7 +2262,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2253,7 +2279,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2270,7 +2296,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2287,7 +2313,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2304,7 +2330,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2321,7 +2347,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2338,7 +2364,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2355,7 +2381,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2372,7 +2398,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2389,7 +2415,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2406,7 +2432,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2423,7 +2449,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2440,7 +2466,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2457,7 +2483,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2474,7 +2500,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2491,7 +2517,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2508,7 +2534,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2525,7 +2551,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2542,7 +2568,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2559,7 +2585,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2576,7 +2602,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2593,7 +2619,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2610,7 +2636,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2627,7 +2653,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2644,7 +2670,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2661,7 +2687,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2678,7 +2704,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2695,7 +2721,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2712,7 +2738,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2729,7 +2755,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2746,7 +2772,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2763,7 +2789,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2780,7 +2806,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2797,7 +2823,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2824,16 +2850,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (18/09/2026 11:57)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,16 +329,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -354,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -362,30 +354,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -685,13 +659,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1300,37 +1274,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1353,13 +1327,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1382,13 +1356,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1417,13 +1391,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1446,13 +1420,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1481,13 +1455,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1516,13 +1490,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1545,13 +1519,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1574,13 +1548,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1603,13 +1577,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1635,13 +1609,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1670,13 +1644,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1699,13 +1673,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1734,13 +1708,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1763,13 +1737,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1798,13 +1772,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1833,13 +1807,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1854,24 +1828,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1888,7 +1862,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1905,7 +1879,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1922,7 +1896,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1939,7 +1913,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1956,7 +1930,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1973,7 +1947,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1990,7 +1964,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2007,7 +1981,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2024,7 +1998,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2041,7 +2015,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2058,7 +2032,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2075,7 +2049,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2092,7 +2066,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2109,7 +2083,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2126,7 +2100,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2143,7 +2117,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2160,7 +2134,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2177,7 +2151,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2194,7 +2168,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2211,7 +2185,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2228,7 +2202,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2245,7 +2219,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2262,7 +2236,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2279,7 +2253,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2296,7 +2270,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2313,7 +2287,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2330,7 +2304,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2347,7 +2321,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2364,7 +2338,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2381,7 +2355,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2398,7 +2372,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2415,7 +2389,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2432,7 +2406,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2449,7 +2423,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2466,7 +2440,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2483,7 +2457,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2500,7 +2474,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2517,7 +2491,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2534,7 +2508,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2551,7 +2525,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2568,7 +2542,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2585,7 +2559,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2602,7 +2576,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2619,7 +2593,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2636,7 +2610,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2653,7 +2627,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2670,7 +2644,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2687,7 +2661,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2704,7 +2678,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2721,7 +2695,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2738,7 +2712,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2755,7 +2729,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2772,7 +2746,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2789,7 +2763,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2806,7 +2780,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2823,7 +2797,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2850,16 +2824,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (18/09/2026 16:38)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,8 +329,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -354,12 +362,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,13 +685,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1274,37 +1300,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1327,13 +1353,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1356,13 +1382,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1391,13 +1417,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1420,13 +1446,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1455,13 +1481,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1490,13 +1516,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1519,13 +1545,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1548,13 +1574,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1577,13 +1603,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1609,13 +1635,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1644,13 +1670,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1673,13 +1699,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1708,13 +1734,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1737,13 +1763,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1772,13 +1798,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1807,13 +1833,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1828,24 +1854,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1862,7 +1888,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1879,7 +1905,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1896,7 +1922,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1913,7 +1939,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1930,7 +1956,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1947,7 +1973,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1964,7 +1990,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -1981,7 +2007,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -1998,7 +2024,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2015,7 +2041,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2032,7 +2058,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2049,7 +2075,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2066,7 +2092,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2083,7 +2109,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2100,7 +2126,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2117,7 +2143,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2134,7 +2160,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2151,7 +2177,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2168,7 +2194,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2185,7 +2211,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2202,7 +2228,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2219,7 +2245,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2236,7 +2262,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2253,7 +2279,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2270,7 +2296,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2287,7 +2313,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2304,7 +2330,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2321,7 +2347,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2338,7 +2364,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2355,7 +2381,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2372,7 +2398,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2389,7 +2415,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2406,7 +2432,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2423,7 +2449,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2440,7 +2466,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2457,7 +2483,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2474,7 +2500,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2491,7 +2517,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2508,7 +2534,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2525,7 +2551,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2542,7 +2568,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2559,7 +2585,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2576,7 +2602,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2593,7 +2619,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2610,7 +2636,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2627,7 +2653,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2644,7 +2670,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2661,7 +2687,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2678,7 +2704,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2695,7 +2721,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2712,7 +2738,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2729,7 +2755,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2746,7 +2772,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2763,7 +2789,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2780,7 +2806,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2797,7 +2823,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2824,16 +2850,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (21/09/2026 14:01)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,16 +329,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -354,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -362,30 +354,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -685,13 +659,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1300,37 +1274,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1353,13 +1327,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1382,13 +1356,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1417,13 +1391,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1446,13 +1420,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1481,13 +1455,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1516,13 +1490,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1545,13 +1519,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1574,13 +1548,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1603,13 +1577,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1635,13 +1609,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1670,13 +1644,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1699,13 +1673,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1734,13 +1708,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1763,13 +1737,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1798,13 +1772,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1833,13 +1807,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1854,24 +1828,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1888,7 +1862,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1905,7 +1879,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1922,7 +1896,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1939,7 +1913,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1956,7 +1930,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1973,7 +1947,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1990,7 +1964,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2007,7 +1981,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2024,7 +1998,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2041,7 +2015,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2058,7 +2032,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2075,7 +2049,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2092,7 +2066,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2109,7 +2083,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2126,7 +2100,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2143,7 +2117,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2160,7 +2134,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2177,7 +2151,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2194,7 +2168,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2211,7 +2185,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2228,7 +2202,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2245,7 +2219,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2262,7 +2236,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2279,7 +2253,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2296,7 +2270,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2313,7 +2287,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2330,7 +2304,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2347,7 +2321,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2364,7 +2338,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2381,7 +2355,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2398,7 +2372,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2415,7 +2389,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2432,7 +2406,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2449,7 +2423,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2466,7 +2440,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2483,7 +2457,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2500,7 +2474,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2517,7 +2491,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2534,7 +2508,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2551,7 +2525,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2568,7 +2542,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2585,7 +2559,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2602,7 +2576,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2619,7 +2593,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2636,7 +2610,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2653,7 +2627,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2670,7 +2644,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2687,7 +2661,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2704,7 +2678,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2721,7 +2695,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2738,7 +2712,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2755,7 +2729,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2772,7 +2746,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2789,7 +2763,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2806,7 +2780,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2823,7 +2797,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2850,16 +2824,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (21/09/2026 14:32)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -329,8 +329,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -354,12 +362,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,13 +685,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1274,37 +1300,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1327,13 +1353,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1356,13 +1382,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1391,13 +1417,13 @@
       <c r="H4" t="s">
         <v>82</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1420,13 +1446,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1455,13 +1481,13 @@
       <c r="H6" t="s">
         <v>83</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1490,13 +1516,13 @@
       <c r="H7" t="s">
         <v>82</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1519,13 +1545,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1548,13 +1574,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1577,13 +1603,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1609,13 +1635,13 @@
       <c r="H11" t="s">
         <v>84</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1644,13 +1670,13 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1673,13 +1699,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1708,13 +1734,13 @@
       <c r="H14" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1737,13 +1763,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1772,13 +1798,13 @@
       <c r="H16" t="s">
         <v>86</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1807,13 +1833,13 @@
       <c r="H17" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1828,24 +1854,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1862,7 +1888,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1879,7 +1905,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1896,7 +1922,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1913,7 +1939,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1930,7 +1956,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1947,7 +1973,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -1964,7 +1990,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -1981,7 +2007,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -1998,7 +2024,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2015,7 +2041,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2032,7 +2058,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2049,7 +2075,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2066,7 +2092,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2083,7 +2109,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2100,7 +2126,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2117,7 +2143,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2134,7 +2160,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2151,7 +2177,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2168,7 +2194,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2185,7 +2211,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2202,7 +2228,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2219,7 +2245,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2236,7 +2262,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2253,7 +2279,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2270,7 +2296,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2287,7 +2313,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2304,7 +2330,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2321,7 +2347,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2338,7 +2364,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2355,7 +2381,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2372,7 +2398,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2389,7 +2415,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2406,7 +2432,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2423,7 +2449,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2440,7 +2466,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2457,7 +2483,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2474,7 +2500,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2491,7 +2517,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2508,7 +2534,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2525,7 +2551,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2542,7 +2568,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2559,7 +2585,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2576,7 +2602,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2593,7 +2619,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2610,7 +2636,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2627,7 +2653,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2644,7 +2670,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2661,7 +2687,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2678,7 +2704,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2695,7 +2721,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2712,7 +2738,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2729,7 +2755,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2746,7 +2772,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2763,7 +2789,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2780,7 +2806,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2797,7 +2823,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2824,16 +2850,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (21/09/2026 20:08)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="103">
   <si>
     <t>linha</t>
   </si>
@@ -100,6 +100,9 @@
     <t>Valor da hora de voo após 1° Reajuste</t>
   </si>
   <si>
+    <t>Aguardando</t>
+  </si>
+  <si>
     <t>Valor Autorizado execução de 08/10/2025 até 08/10/2026</t>
   </si>
   <si>
@@ -131,6 +134,9 @@
   </si>
   <si>
     <t>Valor da hora de voo após 2° Reajuste</t>
+  </si>
+  <si>
+    <t>R$ 4.192,68</t>
   </si>
   <si>
     <t>periodo</t>
@@ -681,7 +687,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1038,164 +1044,164 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B33" t="s">
         <v>27</v>
       </c>
       <c r="C33">
-        <v>9268344.682</v>
+        <v>15854.78</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B34" t="s">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="C34">
-        <v>9171086.169</v>
+        <v>42229.72325</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B35" t="s">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="C35">
-        <v>69457.40325</v>
+        <v>48857.39550000001</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B36" t="s">
-        <v>5</v>
-      </c>
-      <c r="C36">
-        <v>27801.11</v>
+        <v>27</v>
+      </c>
+      <c r="C36" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B37" t="s">
         <v>28</v>
       </c>
       <c r="C37">
-        <v>75617521.51000001</v>
+        <v>9375286.581</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B38" t="s">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="C38">
-        <v>467034.1916</v>
+        <v>9171086.169</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B39" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="C39">
-        <v>809636.1683</v>
+        <v>176399.302</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B40" t="s">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="C40">
-        <v>76894191.87</v>
+        <v>27801.11</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B41" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="C41">
-        <v>7365.68</v>
+        <v>75617521.51000001</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B42" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="C42">
-        <v>7365.68</v>
+        <v>360092.2928</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B43" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="C43">
-        <v>0</v>
+        <v>809636.1683</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B44" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="C44">
-        <v>0</v>
+        <v>76787249.97</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B45" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C45">
-        <v>0</v>
+        <v>7365.68</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B46" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C46">
-        <v>0</v>
+        <v>7365.68</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B47" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C47">
         <v>0</v>
@@ -1203,89 +1209,133 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B48" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="C48">
-        <v>75617521.51000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B49" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="C49">
-        <v>467034.1916</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B50" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="C50">
-        <v>809636.1683</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B51" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="C51">
-        <v>76894191.87</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B52" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C52">
-        <v>86162536.55</v>
+        <v>75617521.51000001</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B53" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="C53">
-        <v>1699.333248</v>
+        <v>360092.2928</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B54" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="C54">
-        <v>0</v>
+        <v>809636.1683</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55">
+        <v>93</v>
+      </c>
+      <c r="B55" t="s">
+        <v>36</v>
+      </c>
+      <c r="C55">
+        <v>76787249.97</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56">
         <v>94</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B56" t="s">
         <v>37</v>
       </c>
-      <c r="C55">
+      <c r="C56">
+        <v>86162536.55</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57">
+        <v>95</v>
+      </c>
+      <c r="B57" t="s">
+        <v>24</v>
+      </c>
+      <c r="C57">
+        <v>1699.333248</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58">
+        <v>96</v>
+      </c>
+      <c r="B58" t="s">
+        <v>25</v>
+      </c>
+      <c r="C58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59">
+        <v>97</v>
+      </c>
+      <c r="B59" t="s">
+        <v>38</v>
+      </c>
+      <c r="C59">
         <v>1699.333248</v>
       </c>
     </row>
@@ -1301,54 +1351,54 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D2">
         <v>748504.24</v>
       </c>
       <c r="E2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F2" t="s">
         <v>3</v>
@@ -1365,19 +1415,19 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D3">
         <v>1110378.24</v>
       </c>
       <c r="E3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F3" t="s">
         <v>3</v>
@@ -1394,28 +1444,28 @@
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D4">
         <v>188246.17</v>
       </c>
       <c r="E4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F4" t="s">
         <v>4</v>
       </c>
       <c r="G4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I4" s="2">
         <v>45768</v>
@@ -1429,19 +1479,19 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D5">
         <v>974557.12</v>
       </c>
       <c r="E5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F5" t="s">
         <v>3</v>
@@ -1458,28 +1508,28 @@
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D6">
         <v>112720.77</v>
       </c>
       <c r="E6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F6" t="s">
         <v>4</v>
       </c>
       <c r="G6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I6" s="2">
         <v>45768</v>
@@ -1493,28 +1543,28 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D7">
         <v>378307.61</v>
       </c>
       <c r="E7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F7" t="s">
         <v>4</v>
       </c>
       <c r="G7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I7" s="2">
         <v>45768</v>
@@ -1528,19 +1578,19 @@
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D8">
         <v>1402001.34</v>
       </c>
       <c r="E8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F8" t="s">
         <v>3</v>
@@ -1557,19 +1607,19 @@
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D9">
         <v>1223702.3</v>
       </c>
       <c r="E9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F9" t="s">
         <v>3</v>
@@ -1586,19 +1636,19 @@
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D10">
         <v>1011677.95</v>
       </c>
       <c r="E10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F10" t="s">
         <v>3</v>
@@ -1615,25 +1665,25 @@
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B11" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D11">
         <v>198332.75</v>
       </c>
       <c r="E11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F11" t="s">
         <v>4</v>
       </c>
       <c r="H11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I11" s="2">
         <v>45809</v>
@@ -1647,28 +1697,28 @@
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D12">
         <v>3315.06</v>
       </c>
       <c r="E12" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F12" t="s">
         <v>4</v>
       </c>
       <c r="G12" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H12" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I12" s="2">
         <v>45768</v>
@@ -1682,19 +1732,19 @@
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D13">
         <v>896744.0600000001</v>
       </c>
       <c r="E13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F13" t="s">
         <v>3</v>
@@ -1711,28 +1761,28 @@
     </row>
     <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D14">
         <v>38718.58</v>
       </c>
       <c r="E14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F14" t="s">
         <v>4</v>
       </c>
       <c r="G14" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="H14" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="I14" s="2">
         <v>45815</v>
@@ -1746,19 +1796,19 @@
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B15" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D15">
         <v>919329.0600000001</v>
       </c>
       <c r="E15" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F15" t="s">
         <v>3</v>
@@ -1775,28 +1825,28 @@
     </row>
     <row r="16" spans="1:11">
       <c r="A16" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D16">
         <v>133124.11</v>
       </c>
       <c r="E16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F16" t="s">
         <v>4</v>
       </c>
       <c r="G16" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H16" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I16" s="2">
         <v>45831</v>
@@ -1810,28 +1860,28 @@
     </row>
     <row r="17" spans="1:11">
       <c r="A17" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D17">
         <v>1528.62</v>
       </c>
       <c r="E17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F17" t="s">
         <v>4</v>
       </c>
       <c r="G17" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H17" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="I17" s="2">
         <v>45833</v>
@@ -1855,19 +1905,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -2851,21 +2901,21 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B2">
         <v>89284800</v>
@@ -2879,7 +2929,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B3">
         <v>8286894.31</v>
@@ -2893,7 +2943,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B4">
         <v>80997905.69</v>
@@ -2907,7 +2957,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B5">
         <v>84788607.68000001</v>
@@ -2921,7 +2971,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B6">
         <v>93075501.98999999</v>
@@ -2935,7 +2985,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D7">
         <v>86162536.55</v>
@@ -2943,7 +2993,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D8">
         <v>95503724.53</v>

</xml_diff>

<commit_message>
Atualização automática: reajuste (22/09/2026 12:31)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,16 +335,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -360,7 +352,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -368,30 +360,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -691,13 +665,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1350,37 +1324,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1403,13 +1377,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1432,13 +1406,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1467,13 +1441,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1496,13 +1470,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1531,13 +1505,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1566,13 +1540,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1595,13 +1569,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1624,13 +1598,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1653,13 +1627,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1685,13 +1659,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1720,13 +1694,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1749,13 +1723,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1784,13 +1758,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1813,13 +1787,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1848,13 +1822,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1883,13 +1857,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1904,24 +1878,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1938,7 +1912,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1955,7 +1929,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1972,7 +1946,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1989,7 +1963,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -2006,7 +1980,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -2023,7 +1997,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2040,7 +2014,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2057,7 +2031,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2074,7 +2048,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2091,7 +2065,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2108,7 +2082,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2125,7 +2099,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2142,7 +2116,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2159,7 +2133,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2176,7 +2150,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2193,7 +2167,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2210,7 +2184,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2227,7 +2201,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2244,7 +2218,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2261,7 +2235,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2278,7 +2252,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2295,7 +2269,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2312,7 +2286,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2329,7 +2303,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2346,7 +2320,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2363,7 +2337,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2380,7 +2354,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2397,7 +2371,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2414,7 +2388,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2431,7 +2405,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2448,7 +2422,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2465,7 +2439,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2482,7 +2456,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2499,7 +2473,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2516,7 +2490,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2533,7 +2507,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2550,7 +2524,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2567,7 +2541,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2584,7 +2558,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2601,7 +2575,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2618,7 +2592,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2635,7 +2609,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2652,7 +2626,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2669,7 +2643,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2686,7 +2660,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2703,7 +2677,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2720,7 +2694,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2737,7 +2711,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2754,7 +2728,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2771,7 +2745,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2788,7 +2762,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2805,7 +2779,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2822,7 +2796,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2839,7 +2813,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2856,7 +2830,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2873,7 +2847,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2900,16 +2874,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (23/09/2026 10:06)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,8 +335,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -352,7 +360,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -360,12 +368,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -665,13 +691,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1324,37 +1350,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1377,13 +1403,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1406,13 +1432,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1441,13 +1467,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1470,13 +1496,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1505,13 +1531,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1540,13 +1566,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1569,13 +1595,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1598,13 +1624,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1627,13 +1653,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1659,13 +1685,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1694,13 +1720,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1723,13 +1749,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1758,13 +1784,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1787,13 +1813,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1822,13 +1848,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1857,13 +1883,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1878,24 +1904,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1912,7 +1938,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1929,7 +1955,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1946,7 +1972,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1963,7 +1989,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1980,7 +2006,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1997,7 +2023,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2014,7 +2040,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2031,7 +2057,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2048,7 +2074,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2065,7 +2091,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2082,7 +2108,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2099,7 +2125,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2116,7 +2142,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2133,7 +2159,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2150,7 +2176,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2167,7 +2193,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2184,7 +2210,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2201,7 +2227,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2218,7 +2244,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2235,7 +2261,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2252,7 +2278,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2269,7 +2295,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2286,7 +2312,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2303,7 +2329,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2320,7 +2346,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2337,7 +2363,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2354,7 +2380,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2371,7 +2397,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2388,7 +2414,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2405,7 +2431,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2422,7 +2448,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2439,7 +2465,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2456,7 +2482,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2473,7 +2499,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2490,7 +2516,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2507,7 +2533,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2524,7 +2550,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2541,7 +2567,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2558,7 +2584,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2575,7 +2601,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2592,7 +2618,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2609,7 +2635,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2626,7 +2652,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2643,7 +2669,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2660,7 +2686,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2677,7 +2703,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2694,7 +2720,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2711,7 +2737,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2728,7 +2754,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2745,7 +2771,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2762,7 +2788,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2779,7 +2805,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2796,7 +2822,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2813,7 +2839,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2830,7 +2856,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2847,7 +2873,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2874,16 +2900,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (23/09/2026 12:28)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,16 +335,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -360,7 +352,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -368,30 +360,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -691,13 +665,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1350,37 +1324,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1403,13 +1377,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1432,13 +1406,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1467,13 +1441,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1496,13 +1470,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1531,13 +1505,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1566,13 +1540,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1595,13 +1569,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1624,13 +1598,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1653,13 +1627,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1685,13 +1659,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1720,13 +1694,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1749,13 +1723,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1784,13 +1758,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1813,13 +1787,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1848,13 +1822,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1883,13 +1857,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1904,24 +1878,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1938,7 +1912,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1955,7 +1929,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1972,7 +1946,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1989,7 +1963,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -2006,7 +1980,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -2023,7 +1997,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2040,7 +2014,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2057,7 +2031,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2074,7 +2048,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2091,7 +2065,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2108,7 +2082,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2125,7 +2099,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2142,7 +2116,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2159,7 +2133,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2176,7 +2150,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2193,7 +2167,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2210,7 +2184,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2227,7 +2201,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2244,7 +2218,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2261,7 +2235,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2278,7 +2252,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2295,7 +2269,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2312,7 +2286,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2329,7 +2303,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2346,7 +2320,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2363,7 +2337,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2380,7 +2354,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2397,7 +2371,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2414,7 +2388,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2431,7 +2405,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2448,7 +2422,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2465,7 +2439,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2482,7 +2456,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2499,7 +2473,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2516,7 +2490,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2533,7 +2507,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2550,7 +2524,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2567,7 +2541,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2584,7 +2558,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2601,7 +2575,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2618,7 +2592,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2635,7 +2609,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2652,7 +2626,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2669,7 +2643,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2686,7 +2660,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2703,7 +2677,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2720,7 +2694,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2737,7 +2711,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2754,7 +2728,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2771,7 +2745,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2788,7 +2762,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2805,7 +2779,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2822,7 +2796,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2839,7 +2813,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2856,7 +2830,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2873,7 +2847,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2900,16 +2874,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (28/09/2026 13:08)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,8 +335,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -352,7 +360,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -360,12 +368,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -665,13 +691,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1324,37 +1350,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1377,13 +1403,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1406,13 +1432,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1441,13 +1467,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1470,13 +1496,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1505,13 +1531,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1540,13 +1566,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1569,13 +1595,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1598,13 +1624,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1627,13 +1653,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1659,13 +1685,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1694,13 +1720,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1723,13 +1749,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1758,13 +1784,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1787,13 +1813,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1822,13 +1848,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1857,13 +1883,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1878,24 +1904,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1912,7 +1938,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1929,7 +1955,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1946,7 +1972,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1963,7 +1989,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1980,7 +2006,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1997,7 +2023,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2014,7 +2040,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2031,7 +2057,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2048,7 +2074,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2065,7 +2091,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2082,7 +2108,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2099,7 +2125,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2116,7 +2142,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2133,7 +2159,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2150,7 +2176,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2167,7 +2193,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2184,7 +2210,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2201,7 +2227,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2218,7 +2244,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2235,7 +2261,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2252,7 +2278,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2269,7 +2295,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2286,7 +2312,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2303,7 +2329,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2320,7 +2346,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2337,7 +2363,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2354,7 +2380,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2371,7 +2397,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2388,7 +2414,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2405,7 +2431,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2422,7 +2448,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2439,7 +2465,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2456,7 +2482,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2473,7 +2499,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2490,7 +2516,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2507,7 +2533,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2524,7 +2550,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2541,7 +2567,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2558,7 +2584,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2575,7 +2601,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2592,7 +2618,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2609,7 +2635,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2626,7 +2652,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2643,7 +2669,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2660,7 +2686,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2677,7 +2703,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2694,7 +2720,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2711,7 +2737,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2728,7 +2754,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2745,7 +2771,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2762,7 +2788,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2779,7 +2805,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2796,7 +2822,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2813,7 +2839,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2830,7 +2856,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2847,7 +2873,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2874,16 +2900,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (28/09/2026 15:36)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,16 +335,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -360,7 +352,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -368,30 +360,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -691,13 +665,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1350,37 +1324,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1403,13 +1377,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1432,13 +1406,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1467,13 +1441,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1496,13 +1470,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1531,13 +1505,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1566,13 +1540,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1595,13 +1569,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1624,13 +1598,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1653,13 +1627,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1685,13 +1659,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1720,13 +1694,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1749,13 +1723,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1784,13 +1758,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1813,13 +1787,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1848,13 +1822,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1883,13 +1857,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1904,24 +1878,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1938,7 +1912,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1955,7 +1929,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1972,7 +1946,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1989,7 +1963,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -2006,7 +1980,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -2023,7 +1997,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2040,7 +2014,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2057,7 +2031,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2074,7 +2048,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2091,7 +2065,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2108,7 +2082,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2125,7 +2099,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2142,7 +2116,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2159,7 +2133,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2176,7 +2150,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2193,7 +2167,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2210,7 +2184,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2227,7 +2201,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2244,7 +2218,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2261,7 +2235,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2278,7 +2252,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2295,7 +2269,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2312,7 +2286,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2329,7 +2303,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2346,7 +2320,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2363,7 +2337,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2380,7 +2354,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2397,7 +2371,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2414,7 +2388,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2431,7 +2405,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2448,7 +2422,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2465,7 +2439,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2482,7 +2456,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2499,7 +2473,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2516,7 +2490,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2533,7 +2507,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2550,7 +2524,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2567,7 +2541,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2584,7 +2558,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2601,7 +2575,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2618,7 +2592,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2635,7 +2609,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2652,7 +2626,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2669,7 +2643,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2686,7 +2660,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2703,7 +2677,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2720,7 +2694,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2737,7 +2711,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2754,7 +2728,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2771,7 +2745,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2788,7 +2762,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2805,7 +2779,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2822,7 +2796,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2839,7 +2813,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2856,7 +2830,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2873,7 +2847,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2900,16 +2874,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (29/09/2026 19:55)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,8 +335,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -352,7 +360,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -360,12 +368,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -665,13 +691,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1324,37 +1350,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1377,13 +1403,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1406,13 +1432,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1441,13 +1467,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1470,13 +1496,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1505,13 +1531,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1540,13 +1566,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1569,13 +1595,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1598,13 +1624,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1627,13 +1653,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1659,13 +1685,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1694,13 +1720,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1723,13 +1749,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1758,13 +1784,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1787,13 +1813,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1822,13 +1848,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1857,13 +1883,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1878,24 +1904,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1912,7 +1938,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1929,7 +1955,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1946,7 +1972,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1963,7 +1989,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1980,7 +2006,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1997,7 +2023,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2014,7 +2040,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2031,7 +2057,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2048,7 +2074,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2065,7 +2091,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2082,7 +2108,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2099,7 +2125,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2116,7 +2142,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2133,7 +2159,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2150,7 +2176,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2167,7 +2193,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2184,7 +2210,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2201,7 +2227,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2218,7 +2244,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2235,7 +2261,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2252,7 +2278,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2269,7 +2295,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2286,7 +2312,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2303,7 +2329,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2320,7 +2346,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2337,7 +2363,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2354,7 +2380,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2371,7 +2397,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2388,7 +2414,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2405,7 +2431,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2422,7 +2448,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2439,7 +2465,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2456,7 +2482,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2473,7 +2499,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2490,7 +2516,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2507,7 +2533,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2524,7 +2550,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2541,7 +2567,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2558,7 +2584,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2575,7 +2601,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2592,7 +2618,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2609,7 +2635,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2626,7 +2652,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2643,7 +2669,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2660,7 +2686,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2677,7 +2703,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2694,7 +2720,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2711,7 +2737,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2728,7 +2754,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2745,7 +2771,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2762,7 +2788,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2779,7 +2805,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2796,7 +2822,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2813,7 +2839,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2830,7 +2856,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2847,7 +2873,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2874,16 +2900,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (30/09/2026 13:49)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,16 +335,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -360,7 +352,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -368,30 +360,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -691,13 +665,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1350,37 +1324,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1403,13 +1377,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1432,13 +1406,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1467,13 +1441,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1496,13 +1470,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1531,13 +1505,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1566,13 +1540,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1595,13 +1569,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1624,13 +1598,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1653,13 +1627,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1685,13 +1659,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1720,13 +1694,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1749,13 +1723,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1784,13 +1758,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1813,13 +1787,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1848,13 +1822,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1883,13 +1857,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1904,24 +1878,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1938,7 +1912,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1955,7 +1929,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1972,7 +1946,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1989,7 +1963,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -2006,7 +1980,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -2023,7 +1997,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2040,7 +2014,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2057,7 +2031,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2074,7 +2048,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2091,7 +2065,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2108,7 +2082,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2125,7 +2099,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2142,7 +2116,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2159,7 +2133,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2176,7 +2150,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2193,7 +2167,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2210,7 +2184,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2227,7 +2201,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2244,7 +2218,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2261,7 +2235,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2278,7 +2252,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2295,7 +2269,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2312,7 +2286,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2329,7 +2303,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2346,7 +2320,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2363,7 +2337,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2380,7 +2354,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2397,7 +2371,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2414,7 +2388,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2431,7 +2405,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2448,7 +2422,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2465,7 +2439,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2482,7 +2456,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2499,7 +2473,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2516,7 +2490,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2533,7 +2507,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2550,7 +2524,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2567,7 +2541,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2584,7 +2558,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2601,7 +2575,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2618,7 +2592,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2635,7 +2609,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2652,7 +2626,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2669,7 +2643,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2686,7 +2660,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2703,7 +2677,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2720,7 +2694,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2737,7 +2711,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2754,7 +2728,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2771,7 +2745,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2788,7 +2762,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2805,7 +2779,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2822,7 +2796,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2839,7 +2813,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2856,7 +2830,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2873,7 +2847,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2900,16 +2874,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (02/10/2026 09:58)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,8 +335,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -352,7 +360,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -360,12 +368,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -665,13 +691,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1324,37 +1350,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1377,13 +1403,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1406,13 +1432,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1441,13 +1467,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1470,13 +1496,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1505,13 +1531,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1540,13 +1566,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1569,13 +1595,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1598,13 +1624,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1627,13 +1653,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1659,13 +1685,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1694,13 +1720,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1723,13 +1749,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1758,13 +1784,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1787,13 +1813,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1822,13 +1848,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1857,13 +1883,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1878,24 +1904,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1912,7 +1938,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1929,7 +1955,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1946,7 +1972,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1963,7 +1989,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1980,7 +2006,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1997,7 +2023,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2014,7 +2040,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2031,7 +2057,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2048,7 +2074,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2065,7 +2091,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2082,7 +2108,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2099,7 +2125,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2116,7 +2142,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2133,7 +2159,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2150,7 +2176,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2167,7 +2193,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2184,7 +2210,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2201,7 +2227,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2218,7 +2244,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2235,7 +2261,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2252,7 +2278,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2269,7 +2295,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2286,7 +2312,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2303,7 +2329,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2320,7 +2346,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2337,7 +2363,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2354,7 +2380,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2371,7 +2397,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2388,7 +2414,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2405,7 +2431,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2422,7 +2448,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2439,7 +2465,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2456,7 +2482,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2473,7 +2499,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2490,7 +2516,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2507,7 +2533,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2524,7 +2550,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2541,7 +2567,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2558,7 +2584,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2575,7 +2601,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2592,7 +2618,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2609,7 +2635,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2626,7 +2652,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2643,7 +2669,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2660,7 +2686,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2677,7 +2703,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2694,7 +2720,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2711,7 +2737,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2728,7 +2754,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2745,7 +2771,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2762,7 +2788,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2779,7 +2805,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2796,7 +2822,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2813,7 +2839,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2830,7 +2856,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2847,7 +2873,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2874,16 +2900,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (02/10/2026 13:38)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,16 +335,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -360,7 +352,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -368,30 +360,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -691,13 +665,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1350,37 +1324,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1403,13 +1377,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1432,13 +1406,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1467,13 +1441,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1496,13 +1470,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1531,13 +1505,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1566,13 +1540,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1595,13 +1569,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1624,13 +1598,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1653,13 +1627,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1685,13 +1659,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1720,13 +1694,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1749,13 +1723,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1784,13 +1758,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1813,13 +1787,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1848,13 +1822,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1883,13 +1857,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1904,24 +1878,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1938,7 +1912,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1955,7 +1929,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1972,7 +1946,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1989,7 +1963,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -2006,7 +1980,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -2023,7 +1997,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2040,7 +2014,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2057,7 +2031,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2074,7 +2048,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2091,7 +2065,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2108,7 +2082,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2125,7 +2099,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2142,7 +2116,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2159,7 +2133,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2176,7 +2150,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2193,7 +2167,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2210,7 +2184,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2227,7 +2201,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2244,7 +2218,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2261,7 +2235,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2278,7 +2252,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2295,7 +2269,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2312,7 +2286,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2329,7 +2303,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2346,7 +2320,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2363,7 +2337,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2380,7 +2354,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2397,7 +2371,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2414,7 +2388,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2431,7 +2405,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2448,7 +2422,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2465,7 +2439,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2482,7 +2456,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2499,7 +2473,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2516,7 +2490,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2533,7 +2507,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2550,7 +2524,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2567,7 +2541,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2584,7 +2558,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2601,7 +2575,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2618,7 +2592,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2635,7 +2609,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2652,7 +2626,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2669,7 +2643,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2686,7 +2660,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2703,7 +2677,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2720,7 +2694,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2737,7 +2711,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2754,7 +2728,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2771,7 +2745,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2788,7 +2762,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2805,7 +2779,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2822,7 +2796,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2839,7 +2813,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2856,7 +2830,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2873,7 +2847,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2900,16 +2874,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (05/10/2026 08:41)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,8 +335,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -352,7 +360,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -360,12 +368,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -665,13 +691,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1324,37 +1350,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1377,13 +1403,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1406,13 +1432,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1441,13 +1467,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1470,13 +1496,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1505,13 +1531,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1540,13 +1566,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1569,13 +1595,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1598,13 +1624,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1627,13 +1653,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1659,13 +1685,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1694,13 +1720,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1723,13 +1749,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1758,13 +1784,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1787,13 +1813,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1822,13 +1848,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1857,13 +1883,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1878,24 +1904,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1912,7 +1938,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1929,7 +1955,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1946,7 +1972,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1963,7 +1989,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1980,7 +2006,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1997,7 +2023,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2014,7 +2040,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2031,7 +2057,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2048,7 +2074,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2065,7 +2091,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2082,7 +2108,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2099,7 +2125,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2116,7 +2142,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2133,7 +2159,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2150,7 +2176,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2167,7 +2193,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2184,7 +2210,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2201,7 +2227,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2218,7 +2244,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2235,7 +2261,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2252,7 +2278,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2269,7 +2295,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2286,7 +2312,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2303,7 +2329,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2320,7 +2346,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2337,7 +2363,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2354,7 +2380,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2371,7 +2397,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2388,7 +2414,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2405,7 +2431,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2422,7 +2448,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2439,7 +2465,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2456,7 +2482,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2473,7 +2499,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2490,7 +2516,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2507,7 +2533,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2524,7 +2550,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2541,7 +2567,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2558,7 +2584,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2575,7 +2601,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2592,7 +2618,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2609,7 +2635,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2626,7 +2652,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2643,7 +2669,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2660,7 +2686,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2677,7 +2703,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2694,7 +2720,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2711,7 +2737,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2728,7 +2754,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2745,7 +2771,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2762,7 +2788,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2779,7 +2805,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2796,7 +2822,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2813,7 +2839,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2830,7 +2856,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2847,7 +2873,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2874,16 +2900,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (06/10/2026 14:11)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,16 +335,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -360,7 +352,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -368,30 +360,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -691,13 +665,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1350,37 +1324,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1403,13 +1377,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1432,13 +1406,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1467,13 +1441,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1496,13 +1470,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1531,13 +1505,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1566,13 +1540,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1595,13 +1569,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1624,13 +1598,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1653,13 +1627,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1685,13 +1659,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1720,13 +1694,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1749,13 +1723,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1784,13 +1758,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1813,13 +1787,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1848,13 +1822,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1883,13 +1857,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1904,24 +1878,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1938,7 +1912,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1955,7 +1929,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1972,7 +1946,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1989,7 +1963,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -2006,7 +1980,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -2023,7 +1997,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2040,7 +2014,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2057,7 +2031,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2074,7 +2048,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2091,7 +2065,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2108,7 +2082,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2125,7 +2099,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2142,7 +2116,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2159,7 +2133,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2176,7 +2150,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2193,7 +2167,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2210,7 +2184,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2227,7 +2201,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2244,7 +2218,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2261,7 +2235,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2278,7 +2252,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2295,7 +2269,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2312,7 +2286,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2329,7 +2303,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2346,7 +2320,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2363,7 +2337,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2380,7 +2354,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2397,7 +2371,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2414,7 +2388,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2431,7 +2405,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2448,7 +2422,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2465,7 +2439,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2482,7 +2456,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2499,7 +2473,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2516,7 +2490,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2533,7 +2507,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2550,7 +2524,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2567,7 +2541,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2584,7 +2558,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2601,7 +2575,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2618,7 +2592,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2635,7 +2609,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2652,7 +2626,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2669,7 +2643,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2686,7 +2660,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2703,7 +2677,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2720,7 +2694,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2737,7 +2711,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2754,7 +2728,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2771,7 +2745,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2788,7 +2762,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2805,7 +2779,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2822,7 +2796,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2839,7 +2813,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2856,7 +2830,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2873,7 +2847,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2900,16 +2874,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (07/10/2026 11:12)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,8 +335,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -352,7 +360,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -360,12 +368,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -665,13 +691,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1324,37 +1350,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1377,13 +1403,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1406,13 +1432,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1441,13 +1467,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1470,13 +1496,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1505,13 +1531,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1540,13 +1566,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1569,13 +1595,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1598,13 +1624,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1627,13 +1653,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1659,13 +1685,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1694,13 +1720,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1723,13 +1749,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1758,13 +1784,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1787,13 +1813,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1822,13 +1848,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1857,13 +1883,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1878,24 +1904,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1912,7 +1938,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1929,7 +1955,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1946,7 +1972,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1963,7 +1989,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1980,7 +2006,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1997,7 +2023,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2014,7 +2040,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2031,7 +2057,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2048,7 +2074,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2065,7 +2091,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2082,7 +2108,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2099,7 +2125,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2116,7 +2142,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2133,7 +2159,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2150,7 +2176,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2167,7 +2193,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2184,7 +2210,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2201,7 +2227,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2218,7 +2244,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2235,7 +2261,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2252,7 +2278,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2269,7 +2295,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2286,7 +2312,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2303,7 +2329,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2320,7 +2346,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2337,7 +2363,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2354,7 +2380,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2371,7 +2397,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2388,7 +2414,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2405,7 +2431,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2422,7 +2448,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2439,7 +2465,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2456,7 +2482,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2473,7 +2499,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2490,7 +2516,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2507,7 +2533,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2524,7 +2550,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2541,7 +2567,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2558,7 +2584,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2575,7 +2601,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2592,7 +2618,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2609,7 +2635,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2626,7 +2652,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2643,7 +2669,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2660,7 +2686,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2677,7 +2703,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2694,7 +2720,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2711,7 +2737,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2728,7 +2754,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2745,7 +2771,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2762,7 +2788,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2779,7 +2805,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2796,7 +2822,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2813,7 +2839,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2830,7 +2856,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2847,7 +2873,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2874,16 +2900,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (07/10/2026 14:48)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,16 +335,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -360,7 +352,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -368,30 +360,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -691,13 +665,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1350,37 +1324,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1403,13 +1377,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1432,13 +1406,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1467,13 +1441,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1496,13 +1470,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1531,13 +1505,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1566,13 +1540,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1595,13 +1569,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1624,13 +1598,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1653,13 +1627,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1685,13 +1659,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1720,13 +1694,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1749,13 +1723,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1784,13 +1758,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1813,13 +1787,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1848,13 +1822,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1883,13 +1857,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1904,24 +1878,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1938,7 +1912,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1955,7 +1929,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1972,7 +1946,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1989,7 +1963,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -2006,7 +1980,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -2023,7 +1997,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2040,7 +2014,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2057,7 +2031,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2074,7 +2048,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2091,7 +2065,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2108,7 +2082,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2125,7 +2099,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2142,7 +2116,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2159,7 +2133,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2176,7 +2150,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2193,7 +2167,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2210,7 +2184,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2227,7 +2201,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2244,7 +2218,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2261,7 +2235,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2278,7 +2252,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2295,7 +2269,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2312,7 +2286,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2329,7 +2303,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2346,7 +2320,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2363,7 +2337,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2380,7 +2354,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2397,7 +2371,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2414,7 +2388,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2431,7 +2405,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2448,7 +2422,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2465,7 +2439,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2482,7 +2456,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2499,7 +2473,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2516,7 +2490,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2533,7 +2507,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2550,7 +2524,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2567,7 +2541,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2584,7 +2558,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2601,7 +2575,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2618,7 +2592,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2635,7 +2609,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2652,7 +2626,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2669,7 +2643,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2686,7 +2660,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2703,7 +2677,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2720,7 +2694,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2737,7 +2711,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2754,7 +2728,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2771,7 +2745,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2788,7 +2762,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2805,7 +2779,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2822,7 +2796,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2839,7 +2813,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2856,7 +2830,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2873,7 +2847,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2900,16 +2874,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (13/10/2026 10:15)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,8 +335,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -352,7 +360,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -360,12 +368,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -665,13 +691,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1324,37 +1350,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1377,13 +1403,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1406,13 +1432,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1441,13 +1467,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1470,13 +1496,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1505,13 +1531,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1540,13 +1566,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1569,13 +1595,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1598,13 +1624,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1627,13 +1653,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1659,13 +1685,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1694,13 +1720,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1723,13 +1749,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1758,13 +1784,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1787,13 +1813,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1822,13 +1848,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1857,13 +1883,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1878,24 +1904,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1912,7 +1938,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1929,7 +1955,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1946,7 +1972,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1963,7 +1989,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1980,7 +2006,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1997,7 +2023,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2014,7 +2040,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2031,7 +2057,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2048,7 +2074,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2065,7 +2091,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2082,7 +2108,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2099,7 +2125,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2116,7 +2142,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2133,7 +2159,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2150,7 +2176,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2167,7 +2193,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2184,7 +2210,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2201,7 +2227,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2218,7 +2244,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2235,7 +2261,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2252,7 +2278,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2269,7 +2295,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2286,7 +2312,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2303,7 +2329,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2320,7 +2346,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2337,7 +2363,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2354,7 +2380,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2371,7 +2397,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2388,7 +2414,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2405,7 +2431,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2422,7 +2448,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2439,7 +2465,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2456,7 +2482,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2473,7 +2499,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2490,7 +2516,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2507,7 +2533,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2524,7 +2550,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2541,7 +2567,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2558,7 +2584,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2575,7 +2601,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2592,7 +2618,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2609,7 +2635,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2626,7 +2652,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2643,7 +2669,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2660,7 +2686,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2677,7 +2703,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2694,7 +2720,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2711,7 +2737,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2728,7 +2754,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2745,7 +2771,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2762,7 +2788,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2779,7 +2805,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2796,7 +2822,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2813,7 +2839,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2830,7 +2856,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2847,7 +2873,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2874,16 +2900,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (13/10/2026 15:10)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,16 +335,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -360,7 +352,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -368,30 +360,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -691,13 +665,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1350,37 +1324,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1403,13 +1377,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1432,13 +1406,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1467,13 +1441,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1496,13 +1470,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1531,13 +1505,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1566,13 +1540,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1595,13 +1569,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1624,13 +1598,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1653,13 +1627,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1685,13 +1659,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1720,13 +1694,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1749,13 +1723,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1784,13 +1758,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1813,13 +1787,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1848,13 +1822,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1883,13 +1857,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1904,24 +1878,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1938,7 +1912,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1955,7 +1929,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1972,7 +1946,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1989,7 +1963,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -2006,7 +1980,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -2023,7 +1997,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2040,7 +2014,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2057,7 +2031,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2074,7 +2048,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2091,7 +2065,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2108,7 +2082,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2125,7 +2099,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2142,7 +2116,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2159,7 +2133,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2176,7 +2150,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2193,7 +2167,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2210,7 +2184,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2227,7 +2201,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2244,7 +2218,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2261,7 +2235,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2278,7 +2252,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2295,7 +2269,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2312,7 +2286,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2329,7 +2303,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2346,7 +2320,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2363,7 +2337,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2380,7 +2354,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2397,7 +2371,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2414,7 +2388,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2431,7 +2405,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2448,7 +2422,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2465,7 +2439,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2482,7 +2456,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2499,7 +2473,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2516,7 +2490,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2533,7 +2507,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2550,7 +2524,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2567,7 +2541,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2584,7 +2558,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2601,7 +2575,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2618,7 +2592,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2635,7 +2609,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2652,7 +2626,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2669,7 +2643,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2686,7 +2660,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2703,7 +2677,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2720,7 +2694,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2737,7 +2711,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2754,7 +2728,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2771,7 +2745,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2788,7 +2762,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2805,7 +2779,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2822,7 +2796,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2839,7 +2813,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2856,7 +2830,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2873,7 +2847,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2900,16 +2874,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (14/10/2026 13:36)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,8 +335,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -352,7 +360,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -360,12 +368,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -665,13 +691,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1324,37 +1350,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1377,13 +1403,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1406,13 +1432,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1441,13 +1467,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1470,13 +1496,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1505,13 +1531,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1540,13 +1566,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1569,13 +1595,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1598,13 +1624,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1627,13 +1653,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1659,13 +1685,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1694,13 +1720,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1723,13 +1749,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1758,13 +1784,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1787,13 +1813,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1822,13 +1848,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1857,13 +1883,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1878,24 +1904,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1912,7 +1938,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1929,7 +1955,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1946,7 +1972,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1963,7 +1989,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1980,7 +2006,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1997,7 +2023,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2014,7 +2040,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2031,7 +2057,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2048,7 +2074,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2065,7 +2091,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2082,7 +2108,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2099,7 +2125,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2116,7 +2142,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2133,7 +2159,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2150,7 +2176,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2167,7 +2193,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2184,7 +2210,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2201,7 +2227,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2218,7 +2244,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2235,7 +2261,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2252,7 +2278,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2269,7 +2295,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2286,7 +2312,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2303,7 +2329,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2320,7 +2346,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2337,7 +2363,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2354,7 +2380,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2371,7 +2397,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2388,7 +2414,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2405,7 +2431,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2422,7 +2448,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2439,7 +2465,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2456,7 +2482,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2473,7 +2499,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2490,7 +2516,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2507,7 +2533,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2524,7 +2550,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2541,7 +2567,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2558,7 +2584,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2575,7 +2601,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2592,7 +2618,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2609,7 +2635,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2626,7 +2652,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2643,7 +2669,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2660,7 +2686,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2677,7 +2703,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2694,7 +2720,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2711,7 +2737,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2728,7 +2754,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2745,7 +2771,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2762,7 +2788,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2779,7 +2805,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2796,7 +2822,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2813,7 +2839,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2830,7 +2856,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2847,7 +2873,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2874,16 +2900,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (15/10/2026 12:36)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,16 +335,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -360,7 +352,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -368,30 +360,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -691,13 +665,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1044,7 +1018,7 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B33" t="s">
         <v>27</v>
@@ -1055,7 +1029,7 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B34" t="s">
         <v>27</v>
@@ -1066,7 +1040,7 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B35" t="s">
         <v>27</v>
@@ -1077,7 +1051,7 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B36" t="s">
         <v>27</v>
@@ -1088,7 +1062,7 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B37" t="s">
         <v>28</v>
@@ -1099,7 +1073,7 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B38" t="s">
         <v>3</v>
@@ -1110,7 +1084,7 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B39" t="s">
         <v>4</v>
@@ -1121,7 +1095,7 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B40" t="s">
         <v>5</v>
@@ -1132,7 +1106,7 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B41" t="s">
         <v>29</v>
@@ -1143,7 +1117,7 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B42" t="s">
         <v>30</v>
@@ -1154,7 +1128,7 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B43" t="s">
         <v>31</v>
@@ -1165,7 +1139,7 @@
     </row>
     <row r="44" spans="1:3">
       <c r="A44">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B44" t="s">
         <v>32</v>
@@ -1176,7 +1150,7 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B45" t="s">
         <v>12</v>
@@ -1187,7 +1161,7 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B46" t="s">
         <v>13</v>
@@ -1198,7 +1172,7 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B47" t="s">
         <v>14</v>
@@ -1209,7 +1183,7 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B48" t="s">
         <v>15</v>
@@ -1220,7 +1194,7 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B49" t="s">
         <v>16</v>
@@ -1231,7 +1205,7 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B50" t="s">
         <v>17</v>
@@ -1242,7 +1216,7 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B51" t="s">
         <v>18</v>
@@ -1253,7 +1227,7 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B52" t="s">
         <v>33</v>
@@ -1264,7 +1238,7 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B53" t="s">
         <v>34</v>
@@ -1275,7 +1249,7 @@
     </row>
     <row r="54" spans="1:3">
       <c r="A54">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B54" t="s">
         <v>35</v>
@@ -1286,7 +1260,7 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B55" t="s">
         <v>36</v>
@@ -1297,7 +1271,7 @@
     </row>
     <row r="56" spans="1:3">
       <c r="A56">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B56" t="s">
         <v>37</v>
@@ -1308,7 +1282,7 @@
     </row>
     <row r="57" spans="1:3">
       <c r="A57">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B57" t="s">
         <v>24</v>
@@ -1319,7 +1293,7 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B58" t="s">
         <v>25</v>
@@ -1330,7 +1304,7 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B59" t="s">
         <v>38</v>
@@ -1350,37 +1324,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1403,13 +1377,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1432,13 +1406,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1467,13 +1441,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1496,13 +1470,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1531,13 +1505,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1566,13 +1540,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1595,13 +1569,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1624,13 +1598,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1653,13 +1627,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1685,13 +1659,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1720,13 +1694,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1749,13 +1723,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1784,13 +1758,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1813,13 +1787,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1848,13 +1822,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1883,13 +1857,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1904,24 +1878,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1938,7 +1912,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1955,7 +1929,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1972,7 +1946,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1989,7 +1963,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -2006,7 +1980,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -2023,7 +1997,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2040,7 +2014,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2057,7 +2031,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2074,7 +2048,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2091,7 +2065,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2108,7 +2082,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2125,7 +2099,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2142,7 +2116,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2159,7 +2133,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2176,7 +2150,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2193,7 +2167,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2210,7 +2184,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2227,7 +2201,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2244,7 +2218,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2261,7 +2235,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2278,7 +2252,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2295,7 +2269,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2312,7 +2286,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2329,7 +2303,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2346,7 +2320,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2363,7 +2337,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2380,7 +2354,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2397,7 +2371,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2414,7 +2388,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2431,7 +2405,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2448,7 +2422,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2465,7 +2439,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2482,7 +2456,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2499,7 +2473,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2516,7 +2490,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2533,7 +2507,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2550,7 +2524,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2567,7 +2541,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2584,7 +2558,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2601,7 +2575,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2618,7 +2592,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2635,7 +2609,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2652,7 +2626,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2669,7 +2643,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2686,7 +2660,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2703,7 +2677,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2720,7 +2694,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2737,7 +2711,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2754,7 +2728,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2771,7 +2745,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2788,7 +2762,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2805,7 +2779,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2822,7 +2796,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2839,7 +2813,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2856,7 +2830,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2873,7 +2847,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2900,16 +2874,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (16/10/2026 12:04)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,8 +335,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -352,7 +360,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -360,12 +368,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -665,13 +691,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1324,37 +1350,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1377,13 +1403,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1406,13 +1432,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1441,13 +1467,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1470,13 +1496,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1505,13 +1531,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1540,13 +1566,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1569,13 +1595,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1598,13 +1624,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1627,13 +1653,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1659,13 +1685,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1694,13 +1720,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1723,13 +1749,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1758,13 +1784,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1787,13 +1813,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1822,13 +1848,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1857,13 +1883,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1878,24 +1904,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1912,7 +1938,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1929,7 +1955,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1946,7 +1972,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1963,7 +1989,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1980,7 +2006,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1997,7 +2023,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2014,7 +2040,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2031,7 +2057,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2048,7 +2074,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2065,7 +2091,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2082,7 +2108,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2099,7 +2125,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2116,7 +2142,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2133,7 +2159,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2150,7 +2176,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2167,7 +2193,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2184,7 +2210,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2201,7 +2227,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2218,7 +2244,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2235,7 +2261,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2252,7 +2278,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2269,7 +2295,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2286,7 +2312,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2303,7 +2329,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2320,7 +2346,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2337,7 +2363,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2354,7 +2380,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2371,7 +2397,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2388,7 +2414,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2405,7 +2431,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2422,7 +2448,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2439,7 +2465,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2456,7 +2482,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2473,7 +2499,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2490,7 +2516,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2507,7 +2533,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2524,7 +2550,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2541,7 +2567,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2558,7 +2584,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2575,7 +2601,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2592,7 +2618,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2609,7 +2635,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2626,7 +2652,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2643,7 +2669,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2660,7 +2686,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2677,7 +2703,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2694,7 +2720,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2711,7 +2737,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2728,7 +2754,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2745,7 +2771,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2762,7 +2788,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2779,7 +2805,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2796,7 +2822,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2813,7 +2839,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2830,7 +2856,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2847,7 +2873,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2874,16 +2900,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (19/10/2026 13:35)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,8 +335,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -352,7 +360,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -360,12 +368,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -665,13 +691,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1324,37 +1350,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1377,13 +1403,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1406,13 +1432,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1441,13 +1467,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1470,13 +1496,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1505,13 +1531,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1540,13 +1566,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1569,13 +1595,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1598,13 +1624,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1627,13 +1653,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1659,13 +1685,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1694,13 +1720,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1723,13 +1749,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1758,13 +1784,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1787,13 +1813,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1822,13 +1848,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1857,13 +1883,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1878,24 +1904,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1912,7 +1938,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1929,7 +1955,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1946,7 +1972,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1963,7 +1989,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1980,7 +2006,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1997,7 +2023,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2014,7 +2040,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2031,7 +2057,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2048,7 +2074,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2065,7 +2091,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2082,7 +2108,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2099,7 +2125,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2116,7 +2142,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2133,7 +2159,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2150,7 +2176,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2167,7 +2193,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2184,7 +2210,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2201,7 +2227,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2218,7 +2244,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2235,7 +2261,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2252,7 +2278,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2269,7 +2295,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2286,7 +2312,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2303,7 +2329,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2320,7 +2346,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2337,7 +2363,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2354,7 +2380,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2371,7 +2397,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2388,7 +2414,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2405,7 +2431,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2422,7 +2448,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2439,7 +2465,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2456,7 +2482,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2473,7 +2499,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2490,7 +2516,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2507,7 +2533,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2524,7 +2550,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2541,7 +2567,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2558,7 +2584,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2575,7 +2601,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2592,7 +2618,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2609,7 +2635,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2626,7 +2652,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2643,7 +2669,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2660,7 +2686,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2677,7 +2703,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2694,7 +2720,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2711,7 +2737,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2728,7 +2754,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2745,7 +2771,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2762,7 +2788,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2779,7 +2805,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2796,7 +2822,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2813,7 +2839,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2830,7 +2856,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2847,7 +2873,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2874,16 +2900,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (19/10/2026 14:28)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,16 +335,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -360,7 +352,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -368,30 +360,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -691,13 +665,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1350,37 +1324,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1403,13 +1377,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1432,13 +1406,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1467,13 +1441,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1496,13 +1470,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1531,13 +1505,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1566,13 +1540,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1595,13 +1569,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1624,13 +1598,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1653,13 +1627,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1685,13 +1659,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1720,13 +1694,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1749,13 +1723,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1784,13 +1758,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1813,13 +1787,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1848,13 +1822,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1883,13 +1857,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1904,24 +1878,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1938,7 +1912,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1955,7 +1929,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1972,7 +1946,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1989,7 +1963,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -2006,7 +1980,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -2023,7 +1997,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2040,7 +2014,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2057,7 +2031,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2074,7 +2048,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2091,7 +2065,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2108,7 +2082,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2125,7 +2099,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2142,7 +2116,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2159,7 +2133,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2176,7 +2150,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2193,7 +2167,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2210,7 +2184,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2227,7 +2201,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2244,7 +2218,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2261,7 +2235,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2278,7 +2252,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2295,7 +2269,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2312,7 +2286,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2329,7 +2303,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2346,7 +2320,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2363,7 +2337,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2380,7 +2354,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2397,7 +2371,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2414,7 +2388,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2431,7 +2405,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2448,7 +2422,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2465,7 +2439,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2482,7 +2456,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2499,7 +2473,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2516,7 +2490,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2533,7 +2507,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2550,7 +2524,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2567,7 +2541,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2584,7 +2558,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2601,7 +2575,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2618,7 +2592,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2635,7 +2609,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2652,7 +2626,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2669,7 +2643,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2686,7 +2660,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2703,7 +2677,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2720,7 +2694,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2737,7 +2711,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2754,7 +2728,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2771,7 +2745,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2788,7 +2762,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2805,7 +2779,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2822,7 +2796,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2839,7 +2813,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2856,7 +2830,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2873,7 +2847,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2900,16 +2874,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (21/10/2026 14:23)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,8 +335,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -352,7 +360,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -360,12 +368,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -665,13 +691,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1324,37 +1350,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1377,13 +1403,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1406,13 +1432,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1441,13 +1467,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1470,13 +1496,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1505,13 +1531,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1540,13 +1566,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1569,13 +1595,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1598,13 +1624,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1627,13 +1653,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1659,13 +1685,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1694,13 +1720,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1723,13 +1749,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1758,13 +1784,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1787,13 +1813,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1822,13 +1848,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1857,13 +1883,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1878,24 +1904,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1912,7 +1938,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1929,7 +1955,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1946,7 +1972,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1963,7 +1989,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1980,7 +2006,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1997,7 +2023,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2014,7 +2040,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2031,7 +2057,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2048,7 +2074,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2065,7 +2091,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2082,7 +2108,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2099,7 +2125,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2116,7 +2142,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2133,7 +2159,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2150,7 +2176,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2167,7 +2193,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2184,7 +2210,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2201,7 +2227,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2218,7 +2244,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2235,7 +2261,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2252,7 +2278,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2269,7 +2295,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2286,7 +2312,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2303,7 +2329,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2320,7 +2346,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2337,7 +2363,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2354,7 +2380,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2371,7 +2397,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2388,7 +2414,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2405,7 +2431,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2422,7 +2448,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2439,7 +2465,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2456,7 +2482,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2473,7 +2499,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2490,7 +2516,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2507,7 +2533,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2524,7 +2550,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2541,7 +2567,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2558,7 +2584,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2575,7 +2601,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2592,7 +2618,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2609,7 +2635,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2626,7 +2652,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2643,7 +2669,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2660,7 +2686,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2677,7 +2703,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2694,7 +2720,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2711,7 +2737,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2728,7 +2754,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2745,7 +2771,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2762,7 +2788,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2779,7 +2805,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2796,7 +2822,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2813,7 +2839,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2830,7 +2856,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2847,7 +2873,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2874,16 +2900,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (22/10/2026 12:54)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,16 +335,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -360,7 +352,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -368,30 +360,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -691,13 +665,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1350,37 +1324,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1403,13 +1377,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1432,13 +1406,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1467,13 +1441,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1496,13 +1470,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1531,13 +1505,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1566,13 +1540,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1595,13 +1569,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1624,13 +1598,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1653,13 +1627,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1685,13 +1659,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1720,13 +1694,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1749,13 +1723,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1784,13 +1758,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1813,13 +1787,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1848,13 +1822,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1883,13 +1857,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1904,24 +1878,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1938,7 +1912,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1955,7 +1929,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1972,7 +1946,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1989,7 +1963,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -2006,7 +1980,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -2023,7 +1997,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2040,7 +2014,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2057,7 +2031,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2074,7 +2048,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2091,7 +2065,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2108,7 +2082,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2125,7 +2099,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2142,7 +2116,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2159,7 +2133,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2176,7 +2150,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2193,7 +2167,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2210,7 +2184,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2227,7 +2201,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2244,7 +2218,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2261,7 +2235,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2278,7 +2252,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2295,7 +2269,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2312,7 +2286,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2329,7 +2303,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2346,7 +2320,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2363,7 +2337,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2380,7 +2354,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2397,7 +2371,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2414,7 +2388,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2431,7 +2405,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2448,7 +2422,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2465,7 +2439,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2482,7 +2456,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2499,7 +2473,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2516,7 +2490,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2533,7 +2507,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2550,7 +2524,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2567,7 +2541,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2584,7 +2558,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2601,7 +2575,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2618,7 +2592,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2635,7 +2609,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2652,7 +2626,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2669,7 +2643,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2686,7 +2660,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2703,7 +2677,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2720,7 +2694,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2737,7 +2711,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2754,7 +2728,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2771,7 +2745,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2788,7 +2762,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2805,7 +2779,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2822,7 +2796,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2839,7 +2813,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2856,7 +2830,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2873,7 +2847,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2900,16 +2874,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (23/10/2026 14:23)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,8 +335,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -352,7 +360,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -360,12 +368,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -665,13 +691,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1324,37 +1350,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1377,13 +1403,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="2">
         <v>45722</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>45740</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45778</v>
       </c>
     </row>
@@ -1406,13 +1432,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
         <v>45722</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>45775</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45806</v>
       </c>
     </row>
@@ -1441,13 +1467,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="2">
         <v>45768</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45791</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45834</v>
       </c>
     </row>
@@ -1470,13 +1496,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="2">
         <v>45753</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>45799</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45844</v>
       </c>
     </row>
@@ -1505,13 +1531,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="2">
         <v>45768</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45814</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1540,13 +1566,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>45768</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45853</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45939</v>
       </c>
     </row>
@@ -1569,13 +1595,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>45783</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45856</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1598,13 +1624,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>45814</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>45856</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45891</v>
       </c>
     </row>
@@ -1627,13 +1653,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="2">
         <v>45844</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45901</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45938</v>
       </c>
     </row>
@@ -1659,13 +1685,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="2">
         <v>45809</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45904</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45935</v>
       </c>
     </row>
@@ -1694,13 +1720,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>45768</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>45910</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45941</v>
       </c>
     </row>
@@ -1723,13 +1749,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>45875</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>45923</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -1758,13 +1784,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="2">
         <v>45815</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>45930</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45991</v>
       </c>
     </row>
@@ -1787,13 +1813,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="2">
         <v>45906</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>45957</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46003</v>
       </c>
     </row>
@@ -1822,13 +1848,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16" s="2">
         <v>45831</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>45968</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -1857,13 +1883,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="1">
+      <c r="I17" s="2">
         <v>45833</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46008</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46066</v>
       </c>
     </row>
@@ -1878,24 +1904,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1912,7 +1938,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1929,7 +1955,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1946,7 +1972,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1963,7 +1989,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -1980,7 +2006,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -1997,7 +2023,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2014,7 +2040,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2031,7 +2057,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2048,7 +2074,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2065,7 +2091,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2082,7 +2108,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2099,7 +2125,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2116,7 +2142,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2133,7 +2159,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2150,7 +2176,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2167,7 +2193,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2184,7 +2210,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2201,7 +2227,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2218,7 +2244,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2235,7 +2261,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2252,7 +2278,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2269,7 +2295,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2286,7 +2312,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2303,7 +2329,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2320,7 +2346,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2337,7 +2363,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2354,7 +2380,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2371,7 +2397,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2388,7 +2414,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2405,7 +2431,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2422,7 +2448,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2439,7 +2465,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2456,7 +2482,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2473,7 +2499,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2490,7 +2516,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2507,7 +2533,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2524,7 +2550,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2541,7 +2567,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2558,7 +2584,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2575,7 +2601,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2592,7 +2618,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2609,7 +2635,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2626,7 +2652,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2643,7 +2669,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2660,7 +2686,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2677,7 +2703,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2694,7 +2720,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2711,7 +2737,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2728,7 +2754,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2745,7 +2771,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2762,7 +2788,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2779,7 +2805,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2796,7 +2822,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2813,7 +2839,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2830,7 +2856,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2847,7 +2873,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2874,16 +2900,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: reajuste (26/10/2026 14:19)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_reajuste_tratada.xlsx
@@ -335,16 +335,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -360,7 +352,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -368,30 +360,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -691,13 +665,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1350,37 +1324,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1403,13 +1377,13 @@
       <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>45722</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>45740</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45778</v>
       </c>
     </row>
@@ -1432,13 +1406,13 @@
       <c r="F3" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>45722</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>45775</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45806</v>
       </c>
     </row>
@@ -1467,13 +1441,13 @@
       <c r="H4" t="s">
         <v>84</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>45768</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>45791</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45834</v>
       </c>
     </row>
@@ -1496,13 +1470,13 @@
       <c r="F5" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>45753</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>45799</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45844</v>
       </c>
     </row>
@@ -1531,13 +1505,13 @@
       <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>45768</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45814</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1566,13 +1540,13 @@
       <c r="H7" t="s">
         <v>84</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>45768</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45853</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45939</v>
       </c>
     </row>
@@ -1595,13 +1569,13 @@
       <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>45783</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45856</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1624,13 +1598,13 @@
       <c r="F9" t="s">
         <v>3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>45814</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>45856</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45891</v>
       </c>
     </row>
@@ -1653,13 +1627,13 @@
       <c r="F10" t="s">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>45844</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45901</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45938</v>
       </c>
     </row>
@@ -1685,13 +1659,13 @@
       <c r="H11" t="s">
         <v>86</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>45809</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45904</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45935</v>
       </c>
     </row>
@@ -1720,13 +1694,13 @@
       <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>45768</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>45910</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45941</v>
       </c>
     </row>
@@ -1749,13 +1723,13 @@
       <c r="F13" t="s">
         <v>3</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>45875</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>45923</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -1784,13 +1758,13 @@
       <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>45815</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>45930</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45991</v>
       </c>
     </row>
@@ -1813,13 +1787,13 @@
       <c r="F15" t="s">
         <v>3</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>45906</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>45957</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46003</v>
       </c>
     </row>
@@ -1848,13 +1822,13 @@
       <c r="H16" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>45831</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>45968</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -1883,13 +1857,13 @@
       <c r="H17" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>45833</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46008</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46066</v>
       </c>
     </row>
@@ -1904,24 +1878,24 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>45689</v>
       </c>
       <c r="B2">
@@ -1938,7 +1912,7 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>45717</v>
       </c>
       <c r="B3">
@@ -1955,7 +1929,7 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>45748</v>
       </c>
       <c r="B4">
@@ -1972,7 +1946,7 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>45778</v>
       </c>
       <c r="B5">
@@ -1989,7 +1963,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>45809</v>
       </c>
       <c r="B6">
@@ -2006,7 +1980,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>45839</v>
       </c>
       <c r="B7">
@@ -2023,7 +1997,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>45870</v>
       </c>
       <c r="B8">
@@ -2040,7 +2014,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>45901</v>
       </c>
       <c r="B9">
@@ -2057,7 +2031,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>45931</v>
       </c>
       <c r="B10">
@@ -2074,7 +2048,7 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>45962</v>
       </c>
       <c r="B11">
@@ -2091,7 +2065,7 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
       <c r="B12">
@@ -2108,7 +2082,7 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>46023</v>
       </c>
       <c r="B13">
@@ -2125,7 +2099,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>46054</v>
       </c>
       <c r="B14">
@@ -2142,7 +2116,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>46082</v>
       </c>
       <c r="B15">
@@ -2159,7 +2133,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>46113</v>
       </c>
       <c r="B16">
@@ -2176,7 +2150,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>46143</v>
       </c>
       <c r="B17">
@@ -2193,7 +2167,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>46174</v>
       </c>
       <c r="B18">
@@ -2210,7 +2184,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>46204</v>
       </c>
       <c r="B19">
@@ -2227,7 +2201,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>46235</v>
       </c>
       <c r="B20">
@@ -2244,7 +2218,7 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>46266</v>
       </c>
       <c r="B21">
@@ -2261,7 +2235,7 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>46296</v>
       </c>
       <c r="B22">
@@ -2278,7 +2252,7 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>46327</v>
       </c>
       <c r="B23">
@@ -2295,7 +2269,7 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>46357</v>
       </c>
       <c r="B24">
@@ -2312,7 +2286,7 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>46388</v>
       </c>
       <c r="B25">
@@ -2329,7 +2303,7 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>46419</v>
       </c>
       <c r="B26">
@@ -2346,7 +2320,7 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>46447</v>
       </c>
       <c r="B27">
@@ -2363,7 +2337,7 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>46478</v>
       </c>
       <c r="B28">
@@ -2380,7 +2354,7 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>46508</v>
       </c>
       <c r="B29">
@@ -2397,7 +2371,7 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>46539</v>
       </c>
       <c r="B30">
@@ -2414,7 +2388,7 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>46569</v>
       </c>
       <c r="B31">
@@ -2431,7 +2405,7 @@
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>46600</v>
       </c>
       <c r="B32">
@@ -2448,7 +2422,7 @@
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>46631</v>
       </c>
       <c r="B33">
@@ -2465,7 +2439,7 @@
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>46661</v>
       </c>
       <c r="B34">
@@ -2482,7 +2456,7 @@
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>46692</v>
       </c>
       <c r="B35">
@@ -2499,7 +2473,7 @@
       </c>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>46722</v>
       </c>
       <c r="B36">
@@ -2516,7 +2490,7 @@
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
+      <c r="A37" s="1">
         <v>46753</v>
       </c>
       <c r="B37">
@@ -2533,7 +2507,7 @@
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="2">
+      <c r="A38" s="1">
         <v>46784</v>
       </c>
       <c r="B38">
@@ -2550,7 +2524,7 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="A39" s="2">
+      <c r="A39" s="1">
         <v>46813</v>
       </c>
       <c r="B39">
@@ -2567,7 +2541,7 @@
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="2">
+      <c r="A40" s="1">
         <v>46844</v>
       </c>
       <c r="B40">
@@ -2584,7 +2558,7 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="2">
+      <c r="A41" s="1">
         <v>46874</v>
       </c>
       <c r="B41">
@@ -2601,7 +2575,7 @@
       </c>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="2">
+      <c r="A42" s="1">
         <v>46905</v>
       </c>
       <c r="B42">
@@ -2618,7 +2592,7 @@
       </c>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="2">
+      <c r="A43" s="1">
         <v>46935</v>
       </c>
       <c r="B43">
@@ -2635,7 +2609,7 @@
       </c>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="2">
+      <c r="A44" s="1">
         <v>46966</v>
       </c>
       <c r="B44">
@@ -2652,7 +2626,7 @@
       </c>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="2">
+      <c r="A45" s="1">
         <v>46997</v>
       </c>
       <c r="B45">
@@ -2669,7 +2643,7 @@
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="2">
+      <c r="A46" s="1">
         <v>47027</v>
       </c>
       <c r="B46">
@@ -2686,7 +2660,7 @@
       </c>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="2">
+      <c r="A47" s="1">
         <v>47058</v>
       </c>
       <c r="B47">
@@ -2703,7 +2677,7 @@
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="2">
+      <c r="A48" s="1">
         <v>47088</v>
       </c>
       <c r="B48">
@@ -2720,7 +2694,7 @@
       </c>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="2">
+      <c r="A49" s="1">
         <v>47119</v>
       </c>
       <c r="B49">
@@ -2737,7 +2711,7 @@
       </c>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="2">
+      <c r="A50" s="1">
         <v>47150</v>
       </c>
       <c r="B50">
@@ -2754,7 +2728,7 @@
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="2">
+      <c r="A51" s="1">
         <v>47178</v>
       </c>
       <c r="B51">
@@ -2771,7 +2745,7 @@
       </c>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="2">
+      <c r="A52" s="1">
         <v>47209</v>
       </c>
       <c r="B52">
@@ -2788,7 +2762,7 @@
       </c>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="2">
+      <c r="A53" s="1">
         <v>47239</v>
       </c>
       <c r="B53">
@@ -2805,7 +2779,7 @@
       </c>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="2">
+      <c r="A54" s="1">
         <v>47270</v>
       </c>
       <c r="B54">
@@ -2822,7 +2796,7 @@
       </c>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="2">
+      <c r="A55" s="1">
         <v>47300</v>
       </c>
       <c r="B55">
@@ -2839,7 +2813,7 @@
       </c>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="2">
+      <c r="A56" s="1">
         <v>47331</v>
       </c>
       <c r="B56">
@@ -2856,7 +2830,7 @@
       </c>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="2">
+      <c r="A57" s="1">
         <v>47362</v>
       </c>
       <c r="B57">
@@ -2873,7 +2847,7 @@
       </c>
     </row>
     <row r="58" spans="1:5">
-      <c r="A58" s="2">
+      <c r="A58" s="1">
         <v>47392</v>
       </c>
       <c r="B58">
@@ -2900,16 +2874,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>